<commit_message>
Refresh camp test data exports
</commit_message>
<xml_diff>
--- a/outputs/test-data/foodpro-camps-ingredient-inventory.xlsx
+++ b/outputs/test-data/foodpro-camps-ingredient-inventory.xlsx
@@ -460,10 +460,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C2" t="str">
         <v>site_abqaiq</v>
@@ -507,10 +507,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C3" t="str">
         <v>site_abqaiq_warehouse</v>
@@ -563,10 +563,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C4" t="str">
         <v>site_modon</v>
@@ -610,10 +610,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C5" t="str">
         <v>site_modon_warehouse</v>
@@ -2205,10 +2205,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C2" t="str">
         <v>inventory_site_abqaiq_ing_basmati_rice</v>
@@ -2270,10 +2270,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C3" t="str">
         <v>inventory_site_abqaiq_ing_chicken_boneless</v>
@@ -2335,10 +2335,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C4" t="str">
         <v>inventory_site_abqaiq_ing_mutton</v>
@@ -2400,10 +2400,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C5" t="str">
         <v>inventory_site_abqaiq_ing_beef_mince</v>
@@ -2465,10 +2465,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C6" t="str">
         <v>inventory_site_abqaiq_ing_penne_pasta</v>
@@ -2530,10 +2530,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C7" t="str">
         <v>inventory_site_abqaiq_ing_spaghetti</v>
@@ -2595,10 +2595,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C8" t="str">
         <v>inventory_site_abqaiq_ing_tomato_puree</v>
@@ -2660,10 +2660,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C9" t="str">
         <v>inventory_site_abqaiq_ing_onion</v>
@@ -2725,10 +2725,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C10" t="str">
         <v>inventory_site_abqaiq_ing_potato</v>
@@ -2790,10 +2790,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C11" t="str">
         <v>inventory_site_abqaiq_ing_mixed_veg</v>
@@ -2855,10 +2855,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C12" t="str">
         <v>inventory_site_abqaiq_ing_capsicum</v>
@@ -2920,10 +2920,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C13" t="str">
         <v>inventory_site_abqaiq_ing_lettuce</v>
@@ -2985,10 +2985,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C14" t="str">
         <v>inventory_site_abqaiq_ing_carrot</v>
@@ -3050,10 +3050,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C15" t="str">
         <v>inventory_site_abqaiq_ing_cucumber</v>
@@ -3115,10 +3115,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C16" t="str">
         <v>inventory_site_abqaiq_ing_yogurt</v>
@@ -3180,10 +3180,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C17" t="str">
         <v>inventory_site_abqaiq_ing_cream</v>
@@ -3245,10 +3245,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C18" t="str">
         <v>inventory_site_abqaiq_ing_mozzarella</v>
@@ -3310,10 +3310,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C19" t="str">
         <v>inventory_site_abqaiq_ing_parmesan</v>
@@ -3375,10 +3375,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C20" t="str">
         <v>inventory_site_abqaiq_ing_flour</v>
@@ -3440,10 +3440,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C21" t="str">
         <v>inventory_site_abqaiq_ing_egg</v>
@@ -3505,10 +3505,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C22" t="str">
         <v>inventory_site_abqaiq_ing_bread_crumbs</v>
@@ -3570,10 +3570,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B23" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C23" t="str">
         <v>inventory_site_abqaiq_ing_olive_oil</v>
@@ -3635,10 +3635,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C24" t="str">
         <v>inventory_site_abqaiq_ing_ghee</v>
@@ -3700,10 +3700,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C25" t="str">
         <v>inventory_site_abqaiq_ing_butter</v>
@@ -3765,10 +3765,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C26" t="str">
         <v>inventory_site_abqaiq_ing_ginger_garlic</v>
@@ -3830,10 +3830,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C27" t="str">
         <v>inventory_site_abqaiq_ing_biryani_masala</v>
@@ -3895,10 +3895,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B28" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C28" t="str">
         <v>inventory_site_abqaiq_ing_garam_masala</v>
@@ -3960,10 +3960,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B29" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C29" t="str">
         <v>inventory_site_abqaiq_ing_italian_herbs</v>
@@ -4025,10 +4025,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B30" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C30" t="str">
         <v>inventory_site_abqaiq_ing_white_sauce_mix</v>
@@ -4090,10 +4090,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B31" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C31" t="str">
         <v>inventory_site_abqaiq_ing_chicken_stock</v>
@@ -4155,10 +4155,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B32" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C32" t="str">
         <v>inventory_site_abqaiq_ing_salt</v>
@@ -4220,10 +4220,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B33" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C33" t="str">
         <v>inventory_site_abqaiq_ing_black_pepper</v>
@@ -4285,10 +4285,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B34" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C34" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_basmati_rice</v>
@@ -4350,10 +4350,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="B35" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.309Z</v>
       </c>
       <c r="C35" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_chicken_boneless</v>
@@ -4415,10 +4415,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B36" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C36" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mutton</v>
@@ -4480,10 +4480,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B37" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C37" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_beef_mince</v>
@@ -4545,10 +4545,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B38" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C38" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_penne_pasta</v>
@@ -4610,10 +4610,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B39" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C39" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_spaghetti</v>
@@ -4675,10 +4675,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B40" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C40" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_tomato_puree</v>
@@ -4740,10 +4740,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B41" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C41" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_onion</v>
@@ -4805,10 +4805,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B42" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C42" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_potato</v>
@@ -4870,10 +4870,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B43" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C43" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mixed_veg</v>
@@ -4935,10 +4935,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B44" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C44" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_capsicum</v>
@@ -5000,10 +5000,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B45" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C45" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_lettuce</v>
@@ -5065,10 +5065,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B46" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C46" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_carrot</v>
@@ -5130,10 +5130,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B47" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C47" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_cucumber</v>
@@ -5195,10 +5195,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B48" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C48" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_yogurt</v>
@@ -5260,10 +5260,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B49" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C49" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_cream</v>
@@ -5325,10 +5325,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B50" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C50" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mozzarella</v>
@@ -5390,10 +5390,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B51" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C51" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_parmesan</v>
@@ -5455,10 +5455,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B52" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C52" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_flour</v>
@@ -5520,10 +5520,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B53" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C53" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_egg</v>
@@ -5585,10 +5585,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B54" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C54" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_bread_crumbs</v>
@@ -5650,10 +5650,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B55" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C55" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_olive_oil</v>
@@ -5715,10 +5715,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B56" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C56" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_ghee</v>
@@ -5780,10 +5780,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B57" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C57" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_butter</v>
@@ -5845,10 +5845,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B58" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C58" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_ginger_garlic</v>
@@ -5910,10 +5910,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B59" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C59" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_biryani_masala</v>
@@ -5975,10 +5975,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B60" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C60" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_garam_masala</v>
@@ -6040,10 +6040,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B61" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C61" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_italian_herbs</v>
@@ -6105,10 +6105,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B62" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C62" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_white_sauce_mix</v>
@@ -6170,10 +6170,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B63" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C63" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_chicken_stock</v>
@@ -6235,10 +6235,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B64" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C64" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_salt</v>
@@ -6300,10 +6300,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B65" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C65" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_black_pepper</v>
@@ -6365,10 +6365,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B66" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C66" t="str">
         <v>inventory_site_modon_ing_basmati_rice</v>
@@ -6430,10 +6430,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B67" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C67" t="str">
         <v>inventory_site_modon_ing_chicken_boneless</v>
@@ -6495,10 +6495,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B68" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C68" t="str">
         <v>inventory_site_modon_ing_mutton</v>
@@ -6560,10 +6560,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B69" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C69" t="str">
         <v>inventory_site_modon_ing_beef_mince</v>
@@ -6625,10 +6625,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B70" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C70" t="str">
         <v>inventory_site_modon_ing_penne_pasta</v>
@@ -6690,10 +6690,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B71" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C71" t="str">
         <v>inventory_site_modon_ing_spaghetti</v>
@@ -6755,10 +6755,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B72" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C72" t="str">
         <v>inventory_site_modon_ing_tomato_puree</v>
@@ -6820,10 +6820,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B73" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C73" t="str">
         <v>inventory_site_modon_ing_onion</v>
@@ -6885,10 +6885,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B74" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C74" t="str">
         <v>inventory_site_modon_ing_potato</v>
@@ -6950,10 +6950,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B75" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C75" t="str">
         <v>inventory_site_modon_ing_mixed_veg</v>
@@ -7015,10 +7015,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B76" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C76" t="str">
         <v>inventory_site_modon_ing_capsicum</v>
@@ -7080,10 +7080,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B77" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C77" t="str">
         <v>inventory_site_modon_ing_lettuce</v>
@@ -7145,10 +7145,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B78" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C78" t="str">
         <v>inventory_site_modon_ing_carrot</v>
@@ -7210,10 +7210,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B79" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C79" t="str">
         <v>inventory_site_modon_ing_cucumber</v>
@@ -7275,10 +7275,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B80" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C80" t="str">
         <v>inventory_site_modon_ing_yogurt</v>
@@ -7340,10 +7340,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B81" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C81" t="str">
         <v>inventory_site_modon_ing_cream</v>
@@ -7405,10 +7405,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B82" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C82" t="str">
         <v>inventory_site_modon_ing_mozzarella</v>
@@ -7470,10 +7470,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B83" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C83" t="str">
         <v>inventory_site_modon_ing_parmesan</v>
@@ -7535,10 +7535,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B84" t="str">
-        <v>2026-05-03T11:13:14.370Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C84" t="str">
         <v>inventory_site_modon_ing_flour</v>
@@ -7600,10 +7600,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B85" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C85" t="str">
         <v>inventory_site_modon_ing_egg</v>
@@ -7665,10 +7665,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B86" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C86" t="str">
         <v>inventory_site_modon_ing_bread_crumbs</v>
@@ -7730,10 +7730,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B87" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C87" t="str">
         <v>inventory_site_modon_ing_olive_oil</v>
@@ -7795,10 +7795,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B88" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C88" t="str">
         <v>inventory_site_modon_ing_ghee</v>
@@ -7860,10 +7860,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B89" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C89" t="str">
         <v>inventory_site_modon_ing_butter</v>
@@ -7925,10 +7925,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B90" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C90" t="str">
         <v>inventory_site_modon_ing_ginger_garlic</v>
@@ -7990,10 +7990,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B91" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C91" t="str">
         <v>inventory_site_modon_ing_biryani_masala</v>
@@ -8055,10 +8055,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B92" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C92" t="str">
         <v>inventory_site_modon_ing_garam_masala</v>
@@ -8120,10 +8120,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B93" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C93" t="str">
         <v>inventory_site_modon_ing_italian_herbs</v>
@@ -8185,10 +8185,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B94" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C94" t="str">
         <v>inventory_site_modon_ing_white_sauce_mix</v>
@@ -8250,10 +8250,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B95" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C95" t="str">
         <v>inventory_site_modon_ing_chicken_stock</v>
@@ -8315,10 +8315,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B96" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C96" t="str">
         <v>inventory_site_modon_ing_salt</v>
@@ -8380,10 +8380,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B97" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C97" t="str">
         <v>inventory_site_modon_ing_black_pepper</v>
@@ -8445,10 +8445,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B98" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C98" t="str">
         <v>inventory_site_modon_warehouse_ing_basmati_rice</v>
@@ -8510,10 +8510,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B99" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C99" t="str">
         <v>inventory_site_modon_warehouse_ing_chicken_boneless</v>
@@ -8575,10 +8575,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B100" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C100" t="str">
         <v>inventory_site_modon_warehouse_ing_mutton</v>
@@ -8640,10 +8640,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B101" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C101" t="str">
         <v>inventory_site_modon_warehouse_ing_beef_mince</v>
@@ -8705,10 +8705,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B102" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C102" t="str">
         <v>inventory_site_modon_warehouse_ing_penne_pasta</v>
@@ -8770,10 +8770,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B103" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C103" t="str">
         <v>inventory_site_modon_warehouse_ing_spaghetti</v>
@@ -8835,10 +8835,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B104" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C104" t="str">
         <v>inventory_site_modon_warehouse_ing_tomato_puree</v>
@@ -8900,10 +8900,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B105" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C105" t="str">
         <v>inventory_site_modon_warehouse_ing_onion</v>
@@ -8965,10 +8965,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B106" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C106" t="str">
         <v>inventory_site_modon_warehouse_ing_potato</v>
@@ -9030,10 +9030,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B107" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C107" t="str">
         <v>inventory_site_modon_warehouse_ing_mixed_veg</v>
@@ -9095,10 +9095,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B108" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C108" t="str">
         <v>inventory_site_modon_warehouse_ing_capsicum</v>
@@ -9160,10 +9160,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B109" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C109" t="str">
         <v>inventory_site_modon_warehouse_ing_lettuce</v>
@@ -9225,10 +9225,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B110" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C110" t="str">
         <v>inventory_site_modon_warehouse_ing_carrot</v>
@@ -9290,10 +9290,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B111" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C111" t="str">
         <v>inventory_site_modon_warehouse_ing_cucumber</v>
@@ -9355,10 +9355,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B112" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C112" t="str">
         <v>inventory_site_modon_warehouse_ing_yogurt</v>
@@ -9420,10 +9420,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B113" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C113" t="str">
         <v>inventory_site_modon_warehouse_ing_cream</v>
@@ -9485,10 +9485,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B114" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C114" t="str">
         <v>inventory_site_modon_warehouse_ing_mozzarella</v>
@@ -9550,10 +9550,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B115" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C115" t="str">
         <v>inventory_site_modon_warehouse_ing_parmesan</v>
@@ -9615,10 +9615,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B116" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C116" t="str">
         <v>inventory_site_modon_warehouse_ing_flour</v>
@@ -9680,10 +9680,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B117" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C117" t="str">
         <v>inventory_site_modon_warehouse_ing_egg</v>
@@ -9745,10 +9745,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B118" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C118" t="str">
         <v>inventory_site_modon_warehouse_ing_bread_crumbs</v>
@@ -9810,10 +9810,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B119" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C119" t="str">
         <v>inventory_site_modon_warehouse_ing_olive_oil</v>
@@ -9875,10 +9875,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B120" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C120" t="str">
         <v>inventory_site_modon_warehouse_ing_ghee</v>
@@ -9940,10 +9940,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B121" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C121" t="str">
         <v>inventory_site_modon_warehouse_ing_butter</v>
@@ -10005,10 +10005,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B122" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C122" t="str">
         <v>inventory_site_modon_warehouse_ing_ginger_garlic</v>
@@ -10070,10 +10070,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B123" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C123" t="str">
         <v>inventory_site_modon_warehouse_ing_biryani_masala</v>
@@ -10135,10 +10135,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B124" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C124" t="str">
         <v>inventory_site_modon_warehouse_ing_garam_masala</v>
@@ -10200,10 +10200,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B125" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C125" t="str">
         <v>inventory_site_modon_warehouse_ing_italian_herbs</v>
@@ -10265,10 +10265,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B126" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C126" t="str">
         <v>inventory_site_modon_warehouse_ing_white_sauce_mix</v>
@@ -10330,10 +10330,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B127" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C127" t="str">
         <v>inventory_site_modon_warehouse_ing_chicken_stock</v>
@@ -10395,10 +10395,10 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B128" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C128" t="str">
         <v>inventory_site_modon_warehouse_ing_salt</v>
@@ -10460,10 +10460,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="B129" t="str">
-        <v>2026-05-03T11:13:14.371Z</v>
+        <v>2026-05-03T11:28:05.310Z</v>
       </c>
       <c r="C129" t="str">
         <v>inventory_site_modon_warehouse_ing_black_pepper</v>

</xml_diff>

<commit_message>
Add role-ready camp test data
</commit_message>
<xml_diff>
--- a/outputs/test-data/foodpro-camps-ingredient-inventory.xlsx
+++ b/outputs/test-data/foodpro-camps-ingredient-inventory.xlsx
@@ -7,6 +7,7 @@
     <sheet name="Ingredients" sheetId="2" r:id="rId2"/>
     <sheet name="Inventory" sheetId="3" r:id="rId3"/>
     <sheet name="Recipes" sheetId="4" r:id="rId4"/>
+    <sheet name="Test Users" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -460,10 +461,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.454Z</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.454Z</v>
       </c>
       <c r="C2" t="str">
         <v>site_abqaiq</v>
@@ -507,10 +508,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.454Z</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.454Z</v>
       </c>
       <c r="C3" t="str">
         <v>site_abqaiq_warehouse</v>
@@ -563,10 +564,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.454Z</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.454Z</v>
       </c>
       <c r="C4" t="str">
         <v>site_modon</v>
@@ -610,10 +611,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.454Z</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.454Z</v>
       </c>
       <c r="C5" t="str">
         <v>site_modon_warehouse</v>
@@ -2205,10 +2206,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="C2" t="str">
         <v>inventory_site_abqaiq_ing_basmati_rice</v>
@@ -2270,10 +2271,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="C3" t="str">
         <v>inventory_site_abqaiq_ing_chicken_boneless</v>
@@ -2335,10 +2336,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="C4" t="str">
         <v>inventory_site_abqaiq_ing_mutton</v>
@@ -2400,10 +2401,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="C5" t="str">
         <v>inventory_site_abqaiq_ing_beef_mince</v>
@@ -2465,10 +2466,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="C6" t="str">
         <v>inventory_site_abqaiq_ing_penne_pasta</v>
@@ -2530,10 +2531,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="C7" t="str">
         <v>inventory_site_abqaiq_ing_spaghetti</v>
@@ -2595,10 +2596,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.450Z</v>
       </c>
       <c r="C8" t="str">
         <v>inventory_site_abqaiq_ing_tomato_puree</v>
@@ -2660,10 +2661,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C9" t="str">
         <v>inventory_site_abqaiq_ing_onion</v>
@@ -2725,10 +2726,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C10" t="str">
         <v>inventory_site_abqaiq_ing_potato</v>
@@ -2790,10 +2791,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C11" t="str">
         <v>inventory_site_abqaiq_ing_mixed_veg</v>
@@ -2855,10 +2856,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C12" t="str">
         <v>inventory_site_abqaiq_ing_capsicum</v>
@@ -2920,10 +2921,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C13" t="str">
         <v>inventory_site_abqaiq_ing_lettuce</v>
@@ -2985,10 +2986,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C14" t="str">
         <v>inventory_site_abqaiq_ing_carrot</v>
@@ -3050,10 +3051,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C15" t="str">
         <v>inventory_site_abqaiq_ing_cucumber</v>
@@ -3115,10 +3116,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C16" t="str">
         <v>inventory_site_abqaiq_ing_yogurt</v>
@@ -3180,10 +3181,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C17" t="str">
         <v>inventory_site_abqaiq_ing_cream</v>
@@ -3245,10 +3246,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C18" t="str">
         <v>inventory_site_abqaiq_ing_mozzarella</v>
@@ -3310,10 +3311,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C19" t="str">
         <v>inventory_site_abqaiq_ing_parmesan</v>
@@ -3375,10 +3376,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C20" t="str">
         <v>inventory_site_abqaiq_ing_flour</v>
@@ -3440,10 +3441,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C21" t="str">
         <v>inventory_site_abqaiq_ing_egg</v>
@@ -3505,10 +3506,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C22" t="str">
         <v>inventory_site_abqaiq_ing_bread_crumbs</v>
@@ -3570,10 +3571,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B23" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C23" t="str">
         <v>inventory_site_abqaiq_ing_olive_oil</v>
@@ -3635,10 +3636,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C24" t="str">
         <v>inventory_site_abqaiq_ing_ghee</v>
@@ -3700,10 +3701,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C25" t="str">
         <v>inventory_site_abqaiq_ing_butter</v>
@@ -3765,10 +3766,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C26" t="str">
         <v>inventory_site_abqaiq_ing_ginger_garlic</v>
@@ -3830,10 +3831,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C27" t="str">
         <v>inventory_site_abqaiq_ing_biryani_masala</v>
@@ -3895,10 +3896,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B28" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C28" t="str">
         <v>inventory_site_abqaiq_ing_garam_masala</v>
@@ -3960,10 +3961,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B29" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C29" t="str">
         <v>inventory_site_abqaiq_ing_italian_herbs</v>
@@ -4025,10 +4026,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B30" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C30" t="str">
         <v>inventory_site_abqaiq_ing_white_sauce_mix</v>
@@ -4090,10 +4091,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B31" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C31" t="str">
         <v>inventory_site_abqaiq_ing_chicken_stock</v>
@@ -4155,10 +4156,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B32" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C32" t="str">
         <v>inventory_site_abqaiq_ing_salt</v>
@@ -4220,10 +4221,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B33" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C33" t="str">
         <v>inventory_site_abqaiq_ing_black_pepper</v>
@@ -4285,10 +4286,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B34" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C34" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_basmati_rice</v>
@@ -4350,10 +4351,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B35" t="str">
-        <v>2026-05-03T11:28:05.309Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C35" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_chicken_boneless</v>
@@ -4415,10 +4416,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B36" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C36" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mutton</v>
@@ -4480,10 +4481,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B37" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C37" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_beef_mince</v>
@@ -4545,10 +4546,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="B38" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.451Z</v>
       </c>
       <c r="C38" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_penne_pasta</v>
@@ -4610,10 +4611,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B39" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C39" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_spaghetti</v>
@@ -4675,10 +4676,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B40" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C40" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_tomato_puree</v>
@@ -4740,10 +4741,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B41" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C41" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_onion</v>
@@ -4805,10 +4806,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B42" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C42" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_potato</v>
@@ -4870,10 +4871,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B43" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C43" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mixed_veg</v>
@@ -4935,10 +4936,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B44" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C44" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_capsicum</v>
@@ -5000,10 +5001,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B45" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C45" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_lettuce</v>
@@ -5065,10 +5066,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B46" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C46" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_carrot</v>
@@ -5130,10 +5131,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B47" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C47" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_cucumber</v>
@@ -5195,10 +5196,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B48" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C48" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_yogurt</v>
@@ -5260,10 +5261,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B49" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C49" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_cream</v>
@@ -5325,10 +5326,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B50" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C50" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mozzarella</v>
@@ -5390,10 +5391,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B51" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C51" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_parmesan</v>
@@ -5455,10 +5456,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B52" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C52" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_flour</v>
@@ -5520,10 +5521,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B53" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C53" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_egg</v>
@@ -5585,10 +5586,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B54" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C54" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_bread_crumbs</v>
@@ -5650,10 +5651,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B55" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C55" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_olive_oil</v>
@@ -5715,10 +5716,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B56" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C56" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_ghee</v>
@@ -5780,10 +5781,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B57" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C57" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_butter</v>
@@ -5845,10 +5846,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B58" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C58" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_ginger_garlic</v>
@@ -5910,10 +5911,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B59" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C59" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_biryani_masala</v>
@@ -5975,10 +5976,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B60" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C60" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_garam_masala</v>
@@ -6040,10 +6041,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B61" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C61" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_italian_herbs</v>
@@ -6105,10 +6106,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B62" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C62" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_white_sauce_mix</v>
@@ -6170,10 +6171,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B63" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C63" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_chicken_stock</v>
@@ -6235,10 +6236,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B64" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C64" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_salt</v>
@@ -6300,10 +6301,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B65" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C65" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_black_pepper</v>
@@ -6365,10 +6366,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B66" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C66" t="str">
         <v>inventory_site_modon_ing_basmati_rice</v>
@@ -6430,10 +6431,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B67" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C67" t="str">
         <v>inventory_site_modon_ing_chicken_boneless</v>
@@ -6495,10 +6496,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B68" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C68" t="str">
         <v>inventory_site_modon_ing_mutton</v>
@@ -6560,10 +6561,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B69" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C69" t="str">
         <v>inventory_site_modon_ing_beef_mince</v>
@@ -6625,10 +6626,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B70" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C70" t="str">
         <v>inventory_site_modon_ing_penne_pasta</v>
@@ -6690,10 +6691,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B71" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C71" t="str">
         <v>inventory_site_modon_ing_spaghetti</v>
@@ -6755,10 +6756,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B72" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C72" t="str">
         <v>inventory_site_modon_ing_tomato_puree</v>
@@ -6820,10 +6821,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B73" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C73" t="str">
         <v>inventory_site_modon_ing_onion</v>
@@ -6885,10 +6886,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B74" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C74" t="str">
         <v>inventory_site_modon_ing_potato</v>
@@ -6950,10 +6951,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B75" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C75" t="str">
         <v>inventory_site_modon_ing_mixed_veg</v>
@@ -7015,10 +7016,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B76" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C76" t="str">
         <v>inventory_site_modon_ing_capsicum</v>
@@ -7080,10 +7081,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B77" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C77" t="str">
         <v>inventory_site_modon_ing_lettuce</v>
@@ -7145,10 +7146,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B78" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C78" t="str">
         <v>inventory_site_modon_ing_carrot</v>
@@ -7210,10 +7211,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B79" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C79" t="str">
         <v>inventory_site_modon_ing_cucumber</v>
@@ -7275,10 +7276,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B80" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C80" t="str">
         <v>inventory_site_modon_ing_yogurt</v>
@@ -7340,10 +7341,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B81" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C81" t="str">
         <v>inventory_site_modon_ing_cream</v>
@@ -7405,10 +7406,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B82" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C82" t="str">
         <v>inventory_site_modon_ing_mozzarella</v>
@@ -7470,10 +7471,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B83" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C83" t="str">
         <v>inventory_site_modon_ing_parmesan</v>
@@ -7535,10 +7536,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B84" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C84" t="str">
         <v>inventory_site_modon_ing_flour</v>
@@ -7600,10 +7601,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B85" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C85" t="str">
         <v>inventory_site_modon_ing_egg</v>
@@ -7665,10 +7666,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B86" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C86" t="str">
         <v>inventory_site_modon_ing_bread_crumbs</v>
@@ -7730,10 +7731,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B87" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C87" t="str">
         <v>inventory_site_modon_ing_olive_oil</v>
@@ -7795,10 +7796,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B88" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C88" t="str">
         <v>inventory_site_modon_ing_ghee</v>
@@ -7860,10 +7861,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B89" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C89" t="str">
         <v>inventory_site_modon_ing_butter</v>
@@ -7925,10 +7926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B90" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C90" t="str">
         <v>inventory_site_modon_ing_ginger_garlic</v>
@@ -7990,10 +7991,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B91" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C91" t="str">
         <v>inventory_site_modon_ing_biryani_masala</v>
@@ -8055,10 +8056,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B92" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C92" t="str">
         <v>inventory_site_modon_ing_garam_masala</v>
@@ -8120,10 +8121,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B93" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C93" t="str">
         <v>inventory_site_modon_ing_italian_herbs</v>
@@ -8185,10 +8186,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B94" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C94" t="str">
         <v>inventory_site_modon_ing_white_sauce_mix</v>
@@ -8250,10 +8251,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B95" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C95" t="str">
         <v>inventory_site_modon_ing_chicken_stock</v>
@@ -8315,10 +8316,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B96" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C96" t="str">
         <v>inventory_site_modon_ing_salt</v>
@@ -8380,10 +8381,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B97" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C97" t="str">
         <v>inventory_site_modon_ing_black_pepper</v>
@@ -8445,10 +8446,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B98" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C98" t="str">
         <v>inventory_site_modon_warehouse_ing_basmati_rice</v>
@@ -8510,10 +8511,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B99" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C99" t="str">
         <v>inventory_site_modon_warehouse_ing_chicken_boneless</v>
@@ -8575,10 +8576,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B100" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C100" t="str">
         <v>inventory_site_modon_warehouse_ing_mutton</v>
@@ -8640,10 +8641,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B101" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C101" t="str">
         <v>inventory_site_modon_warehouse_ing_beef_mince</v>
@@ -8705,10 +8706,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B102" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C102" t="str">
         <v>inventory_site_modon_warehouse_ing_penne_pasta</v>
@@ -8770,10 +8771,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="B103" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.452Z</v>
       </c>
       <c r="C103" t="str">
         <v>inventory_site_modon_warehouse_ing_spaghetti</v>
@@ -8835,10 +8836,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B104" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C104" t="str">
         <v>inventory_site_modon_warehouse_ing_tomato_puree</v>
@@ -8900,10 +8901,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B105" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C105" t="str">
         <v>inventory_site_modon_warehouse_ing_onion</v>
@@ -8965,10 +8966,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B106" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C106" t="str">
         <v>inventory_site_modon_warehouse_ing_potato</v>
@@ -9030,10 +9031,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B107" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C107" t="str">
         <v>inventory_site_modon_warehouse_ing_mixed_veg</v>
@@ -9095,10 +9096,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B108" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C108" t="str">
         <v>inventory_site_modon_warehouse_ing_capsicum</v>
@@ -9160,10 +9161,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B109" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C109" t="str">
         <v>inventory_site_modon_warehouse_ing_lettuce</v>
@@ -9225,10 +9226,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B110" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C110" t="str">
         <v>inventory_site_modon_warehouse_ing_carrot</v>
@@ -9290,10 +9291,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B111" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C111" t="str">
         <v>inventory_site_modon_warehouse_ing_cucumber</v>
@@ -9355,10 +9356,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B112" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C112" t="str">
         <v>inventory_site_modon_warehouse_ing_yogurt</v>
@@ -9420,10 +9421,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B113" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C113" t="str">
         <v>inventory_site_modon_warehouse_ing_cream</v>
@@ -9485,10 +9486,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B114" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C114" t="str">
         <v>inventory_site_modon_warehouse_ing_mozzarella</v>
@@ -9550,10 +9551,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B115" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C115" t="str">
         <v>inventory_site_modon_warehouse_ing_parmesan</v>
@@ -9615,10 +9616,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B116" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C116" t="str">
         <v>inventory_site_modon_warehouse_ing_flour</v>
@@ -9680,10 +9681,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B117" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C117" t="str">
         <v>inventory_site_modon_warehouse_ing_egg</v>
@@ -9745,10 +9746,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B118" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C118" t="str">
         <v>inventory_site_modon_warehouse_ing_bread_crumbs</v>
@@ -9810,10 +9811,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B119" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C119" t="str">
         <v>inventory_site_modon_warehouse_ing_olive_oil</v>
@@ -9875,10 +9876,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B120" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C120" t="str">
         <v>inventory_site_modon_warehouse_ing_ghee</v>
@@ -9940,10 +9941,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B121" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C121" t="str">
         <v>inventory_site_modon_warehouse_ing_butter</v>
@@ -10005,10 +10006,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B122" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C122" t="str">
         <v>inventory_site_modon_warehouse_ing_ginger_garlic</v>
@@ -10070,10 +10071,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B123" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C123" t="str">
         <v>inventory_site_modon_warehouse_ing_biryani_masala</v>
@@ -10135,10 +10136,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B124" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C124" t="str">
         <v>inventory_site_modon_warehouse_ing_garam_masala</v>
@@ -10200,10 +10201,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B125" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C125" t="str">
         <v>inventory_site_modon_warehouse_ing_italian_herbs</v>
@@ -10265,10 +10266,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B126" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C126" t="str">
         <v>inventory_site_modon_warehouse_ing_white_sauce_mix</v>
@@ -10330,10 +10331,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B127" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C127" t="str">
         <v>inventory_site_modon_warehouse_ing_chicken_stock</v>
@@ -10395,10 +10396,10 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B128" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C128" t="str">
         <v>inventory_site_modon_warehouse_ing_salt</v>
@@ -10460,10 +10461,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="B129" t="str">
-        <v>2026-05-03T11:28:05.310Z</v>
+        <v>2026-05-03T13:12:55.453Z</v>
       </c>
       <c r="C129" t="str">
         <v>inventory_site_modon_warehouse_ing_black_pepper</v>
@@ -10792,4 +10793,115 @@
     <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>email</v>
+      </c>
+      <c r="B1" t="str">
+        <v>full_name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>role</v>
+      </c>
+      <c r="D1" t="str">
+        <v>password</v>
+      </c>
+      <c r="E1" t="str">
+        <v>primary_site</v>
+      </c>
+      <c r="F1" t="str">
+        <v>allowed_sites</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>abqaiq.manager@foodpro.test</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ABQAIQ Camp Manager</v>
+      </c>
+      <c r="C2" t="str">
+        <v>manager</v>
+      </c>
+      <c r="D2" t="str">
+        <v>FoodPro@2030</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ABQAIQ CAMP</v>
+      </c>
+      <c r="F2" t="str">
+        <v>ABQAIQ CAMP, ABQAIQ CAMP WAREHOUSE</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>abqaiq.storekeeper@foodpro.test</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ABQAIQ Storekeeper</v>
+      </c>
+      <c r="C3" t="str">
+        <v>user</v>
+      </c>
+      <c r="D3" t="str">
+        <v>FoodPro@2030</v>
+      </c>
+      <c r="E3" t="str">
+        <v>ABQAIQ CAMP</v>
+      </c>
+      <c r="F3" t="str">
+        <v>ABQAIQ CAMP, ABQAIQ CAMP WAREHOUSE</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>modon.manager@foodpro.test</v>
+      </c>
+      <c r="B4" t="str">
+        <v>MODON Camp Manager</v>
+      </c>
+      <c r="C4" t="str">
+        <v>manager</v>
+      </c>
+      <c r="D4" t="str">
+        <v>FoodPro@2030</v>
+      </c>
+      <c r="E4" t="str">
+        <v>MODON CAMP</v>
+      </c>
+      <c r="F4" t="str">
+        <v>MODON CAMP, MODON CAMP WAREHOUSE</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>modon.storekeeper@foodpro.test</v>
+      </c>
+      <c r="B5" t="str">
+        <v>MODON Storekeeper</v>
+      </c>
+      <c r="C5" t="str">
+        <v>user</v>
+      </c>
+      <c r="D5" t="str">
+        <v>FoodPro@2030</v>
+      </c>
+      <c r="E5" t="str">
+        <v>MODON CAMP</v>
+      </c>
+      <c r="F5" t="str">
+        <v>MODON CAMP, MODON CAMP WAREHOUSE</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh injected camp test exports
</commit_message>
<xml_diff>
--- a/outputs/test-data/foodpro-camps-ingredient-inventory.xlsx
+++ b/outputs/test-data/foodpro-camps-ingredient-inventory.xlsx
@@ -461,10 +461,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-05-03T13:12:55.454Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-03T13:12:55.454Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C2" t="str">
         <v>site_abqaiq</v>
@@ -508,10 +508,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-05-03T13:12:55.454Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-03T13:12:55.454Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C3" t="str">
         <v>site_abqaiq_warehouse</v>
@@ -564,10 +564,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-05-03T13:12:55.454Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-03T13:12:55.454Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C4" t="str">
         <v>site_modon</v>
@@ -611,10 +611,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-05-03T13:12:55.454Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-05-03T13:12:55.454Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C5" t="str">
         <v>site_modon_warehouse</v>
@@ -2206,10 +2206,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C2" t="str">
         <v>inventory_site_abqaiq_ing_basmati_rice</v>
@@ -2271,10 +2271,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C3" t="str">
         <v>inventory_site_abqaiq_ing_chicken_boneless</v>
@@ -2336,10 +2336,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C4" t="str">
         <v>inventory_site_abqaiq_ing_mutton</v>
@@ -2401,10 +2401,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C5" t="str">
         <v>inventory_site_abqaiq_ing_beef_mince</v>
@@ -2466,10 +2466,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C6" t="str">
         <v>inventory_site_abqaiq_ing_penne_pasta</v>
@@ -2531,10 +2531,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C7" t="str">
         <v>inventory_site_abqaiq_ing_spaghetti</v>
@@ -2596,10 +2596,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-05-03T13:12:55.450Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C8" t="str">
         <v>inventory_site_abqaiq_ing_tomato_puree</v>
@@ -2661,10 +2661,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C9" t="str">
         <v>inventory_site_abqaiq_ing_onion</v>
@@ -2726,10 +2726,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C10" t="str">
         <v>inventory_site_abqaiq_ing_potato</v>
@@ -2791,10 +2791,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C11" t="str">
         <v>inventory_site_abqaiq_ing_mixed_veg</v>
@@ -2856,10 +2856,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C12" t="str">
         <v>inventory_site_abqaiq_ing_capsicum</v>
@@ -2921,10 +2921,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C13" t="str">
         <v>inventory_site_abqaiq_ing_lettuce</v>
@@ -2986,10 +2986,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C14" t="str">
         <v>inventory_site_abqaiq_ing_carrot</v>
@@ -3051,10 +3051,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C15" t="str">
         <v>inventory_site_abqaiq_ing_cucumber</v>
@@ -3116,10 +3116,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C16" t="str">
         <v>inventory_site_abqaiq_ing_yogurt</v>
@@ -3181,10 +3181,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C17" t="str">
         <v>inventory_site_abqaiq_ing_cream</v>
@@ -3246,10 +3246,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C18" t="str">
         <v>inventory_site_abqaiq_ing_mozzarella</v>
@@ -3311,10 +3311,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C19" t="str">
         <v>inventory_site_abqaiq_ing_parmesan</v>
@@ -3376,10 +3376,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C20" t="str">
         <v>inventory_site_abqaiq_ing_flour</v>
@@ -3441,10 +3441,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C21" t="str">
         <v>inventory_site_abqaiq_ing_egg</v>
@@ -3506,10 +3506,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C22" t="str">
         <v>inventory_site_abqaiq_ing_bread_crumbs</v>
@@ -3571,10 +3571,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B23" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C23" t="str">
         <v>inventory_site_abqaiq_ing_olive_oil</v>
@@ -3636,10 +3636,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B24" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C24" t="str">
         <v>inventory_site_abqaiq_ing_ghee</v>
@@ -3701,10 +3701,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B25" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C25" t="str">
         <v>inventory_site_abqaiq_ing_butter</v>
@@ -3766,10 +3766,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B26" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C26" t="str">
         <v>inventory_site_abqaiq_ing_ginger_garlic</v>
@@ -3831,10 +3831,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B27" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C27" t="str">
         <v>inventory_site_abqaiq_ing_biryani_masala</v>
@@ -3896,10 +3896,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B28" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C28" t="str">
         <v>inventory_site_abqaiq_ing_garam_masala</v>
@@ -3961,10 +3961,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B29" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C29" t="str">
         <v>inventory_site_abqaiq_ing_italian_herbs</v>
@@ -4026,10 +4026,10 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B30" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C30" t="str">
         <v>inventory_site_abqaiq_ing_white_sauce_mix</v>
@@ -4091,10 +4091,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B31" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C31" t="str">
         <v>inventory_site_abqaiq_ing_chicken_stock</v>
@@ -4156,10 +4156,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B32" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C32" t="str">
         <v>inventory_site_abqaiq_ing_salt</v>
@@ -4221,10 +4221,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B33" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C33" t="str">
         <v>inventory_site_abqaiq_ing_black_pepper</v>
@@ -4286,10 +4286,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B34" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C34" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_basmati_rice</v>
@@ -4351,10 +4351,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B35" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C35" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_chicken_boneless</v>
@@ -4416,10 +4416,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B36" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C36" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mutton</v>
@@ -4481,10 +4481,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B37" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C37" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_beef_mince</v>
@@ -4546,10 +4546,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B38" t="str">
-        <v>2026-05-03T13:12:55.451Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C38" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_penne_pasta</v>
@@ -4611,10 +4611,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B39" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C39" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_spaghetti</v>
@@ -4676,10 +4676,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B40" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C40" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_tomato_puree</v>
@@ -4741,10 +4741,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B41" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C41" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_onion</v>
@@ -4806,10 +4806,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B42" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C42" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_potato</v>
@@ -4871,10 +4871,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B43" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C43" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mixed_veg</v>
@@ -4936,10 +4936,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B44" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C44" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_capsicum</v>
@@ -5001,10 +5001,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B45" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C45" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_lettuce</v>
@@ -5066,10 +5066,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B46" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C46" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_carrot</v>
@@ -5131,10 +5131,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B47" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C47" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_cucumber</v>
@@ -5196,10 +5196,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B48" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C48" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_yogurt</v>
@@ -5261,10 +5261,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B49" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C49" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_cream</v>
@@ -5326,10 +5326,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B50" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C50" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_mozzarella</v>
@@ -5391,10 +5391,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B51" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C51" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_parmesan</v>
@@ -5456,10 +5456,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B52" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C52" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_flour</v>
@@ -5521,10 +5521,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B53" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C53" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_egg</v>
@@ -5586,10 +5586,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B54" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C54" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_bread_crumbs</v>
@@ -5651,10 +5651,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B55" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C55" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_olive_oil</v>
@@ -5716,10 +5716,10 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B56" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C56" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_ghee</v>
@@ -5781,10 +5781,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B57" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C57" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_butter</v>
@@ -5846,10 +5846,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B58" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C58" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_ginger_garlic</v>
@@ -5911,10 +5911,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B59" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C59" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_biryani_masala</v>
@@ -5976,10 +5976,10 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B60" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C60" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_garam_masala</v>
@@ -6041,10 +6041,10 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B61" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C61" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_italian_herbs</v>
@@ -6106,10 +6106,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B62" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C62" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_white_sauce_mix</v>
@@ -6171,10 +6171,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B63" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C63" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_chicken_stock</v>
@@ -6236,10 +6236,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B64" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C64" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_salt</v>
@@ -6301,10 +6301,10 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B65" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C65" t="str">
         <v>inventory_site_abqaiq_warehouse_ing_black_pepper</v>
@@ -6366,10 +6366,10 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B66" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C66" t="str">
         <v>inventory_site_modon_ing_basmati_rice</v>
@@ -6431,10 +6431,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B67" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C67" t="str">
         <v>inventory_site_modon_ing_chicken_boneless</v>
@@ -6496,10 +6496,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B68" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C68" t="str">
         <v>inventory_site_modon_ing_mutton</v>
@@ -6561,10 +6561,10 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B69" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C69" t="str">
         <v>inventory_site_modon_ing_beef_mince</v>
@@ -6626,10 +6626,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B70" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C70" t="str">
         <v>inventory_site_modon_ing_penne_pasta</v>
@@ -6691,10 +6691,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B71" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C71" t="str">
         <v>inventory_site_modon_ing_spaghetti</v>
@@ -6756,10 +6756,10 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B72" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C72" t="str">
         <v>inventory_site_modon_ing_tomato_puree</v>
@@ -6821,10 +6821,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B73" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C73" t="str">
         <v>inventory_site_modon_ing_onion</v>
@@ -6886,10 +6886,10 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B74" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C74" t="str">
         <v>inventory_site_modon_ing_potato</v>
@@ -6951,10 +6951,10 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B75" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C75" t="str">
         <v>inventory_site_modon_ing_mixed_veg</v>
@@ -7016,10 +7016,10 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B76" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C76" t="str">
         <v>inventory_site_modon_ing_capsicum</v>
@@ -7081,10 +7081,10 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B77" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C77" t="str">
         <v>inventory_site_modon_ing_lettuce</v>
@@ -7146,10 +7146,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B78" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C78" t="str">
         <v>inventory_site_modon_ing_carrot</v>
@@ -7211,10 +7211,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B79" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C79" t="str">
         <v>inventory_site_modon_ing_cucumber</v>
@@ -7276,10 +7276,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B80" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C80" t="str">
         <v>inventory_site_modon_ing_yogurt</v>
@@ -7341,10 +7341,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B81" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C81" t="str">
         <v>inventory_site_modon_ing_cream</v>
@@ -7406,10 +7406,10 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B82" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C82" t="str">
         <v>inventory_site_modon_ing_mozzarella</v>
@@ -7471,10 +7471,10 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B83" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C83" t="str">
         <v>inventory_site_modon_ing_parmesan</v>
@@ -7536,10 +7536,10 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B84" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C84" t="str">
         <v>inventory_site_modon_ing_flour</v>
@@ -7601,10 +7601,10 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B85" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C85" t="str">
         <v>inventory_site_modon_ing_egg</v>
@@ -7666,10 +7666,10 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="B86" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.845Z</v>
       </c>
       <c r="C86" t="str">
         <v>inventory_site_modon_ing_bread_crumbs</v>
@@ -7731,10 +7731,10 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B87" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C87" t="str">
         <v>inventory_site_modon_ing_olive_oil</v>
@@ -7796,10 +7796,10 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B88" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C88" t="str">
         <v>inventory_site_modon_ing_ghee</v>
@@ -7861,10 +7861,10 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B89" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C89" t="str">
         <v>inventory_site_modon_ing_butter</v>
@@ -7926,10 +7926,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B90" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C90" t="str">
         <v>inventory_site_modon_ing_ginger_garlic</v>
@@ -7991,10 +7991,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B91" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C91" t="str">
         <v>inventory_site_modon_ing_biryani_masala</v>
@@ -8056,10 +8056,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B92" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C92" t="str">
         <v>inventory_site_modon_ing_garam_masala</v>
@@ -8121,10 +8121,10 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B93" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C93" t="str">
         <v>inventory_site_modon_ing_italian_herbs</v>
@@ -8186,10 +8186,10 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B94" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C94" t="str">
         <v>inventory_site_modon_ing_white_sauce_mix</v>
@@ -8251,10 +8251,10 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B95" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C95" t="str">
         <v>inventory_site_modon_ing_chicken_stock</v>
@@ -8316,10 +8316,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B96" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C96" t="str">
         <v>inventory_site_modon_ing_salt</v>
@@ -8381,10 +8381,10 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B97" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C97" t="str">
         <v>inventory_site_modon_ing_black_pepper</v>
@@ -8446,10 +8446,10 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B98" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C98" t="str">
         <v>inventory_site_modon_warehouse_ing_basmati_rice</v>
@@ -8511,10 +8511,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B99" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C99" t="str">
         <v>inventory_site_modon_warehouse_ing_chicken_boneless</v>
@@ -8576,10 +8576,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B100" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C100" t="str">
         <v>inventory_site_modon_warehouse_ing_mutton</v>
@@ -8641,10 +8641,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B101" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C101" t="str">
         <v>inventory_site_modon_warehouse_ing_beef_mince</v>
@@ -8706,10 +8706,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B102" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C102" t="str">
         <v>inventory_site_modon_warehouse_ing_penne_pasta</v>
@@ -8771,10 +8771,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B103" t="str">
-        <v>2026-05-03T13:12:55.452Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C103" t="str">
         <v>inventory_site_modon_warehouse_ing_spaghetti</v>
@@ -8836,10 +8836,10 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B104" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C104" t="str">
         <v>inventory_site_modon_warehouse_ing_tomato_puree</v>
@@ -8901,10 +8901,10 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B105" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C105" t="str">
         <v>inventory_site_modon_warehouse_ing_onion</v>
@@ -8966,10 +8966,10 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B106" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C106" t="str">
         <v>inventory_site_modon_warehouse_ing_potato</v>
@@ -9031,10 +9031,10 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B107" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C107" t="str">
         <v>inventory_site_modon_warehouse_ing_mixed_veg</v>
@@ -9096,10 +9096,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B108" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C108" t="str">
         <v>inventory_site_modon_warehouse_ing_capsicum</v>
@@ -9161,10 +9161,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B109" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C109" t="str">
         <v>inventory_site_modon_warehouse_ing_lettuce</v>
@@ -9226,10 +9226,10 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B110" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C110" t="str">
         <v>inventory_site_modon_warehouse_ing_carrot</v>
@@ -9291,10 +9291,10 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B111" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C111" t="str">
         <v>inventory_site_modon_warehouse_ing_cucumber</v>
@@ -9356,10 +9356,10 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B112" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C112" t="str">
         <v>inventory_site_modon_warehouse_ing_yogurt</v>
@@ -9421,10 +9421,10 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B113" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C113" t="str">
         <v>inventory_site_modon_warehouse_ing_cream</v>
@@ -9486,10 +9486,10 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B114" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C114" t="str">
         <v>inventory_site_modon_warehouse_ing_mozzarella</v>
@@ -9551,10 +9551,10 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B115" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C115" t="str">
         <v>inventory_site_modon_warehouse_ing_parmesan</v>
@@ -9616,10 +9616,10 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B116" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C116" t="str">
         <v>inventory_site_modon_warehouse_ing_flour</v>
@@ -9681,10 +9681,10 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B117" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C117" t="str">
         <v>inventory_site_modon_warehouse_ing_egg</v>
@@ -9746,10 +9746,10 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B118" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C118" t="str">
         <v>inventory_site_modon_warehouse_ing_bread_crumbs</v>
@@ -9811,10 +9811,10 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B119" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C119" t="str">
         <v>inventory_site_modon_warehouse_ing_olive_oil</v>
@@ -9876,10 +9876,10 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B120" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C120" t="str">
         <v>inventory_site_modon_warehouse_ing_ghee</v>
@@ -9941,10 +9941,10 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B121" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C121" t="str">
         <v>inventory_site_modon_warehouse_ing_butter</v>
@@ -10006,10 +10006,10 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B122" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C122" t="str">
         <v>inventory_site_modon_warehouse_ing_ginger_garlic</v>
@@ -10071,10 +10071,10 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B123" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C123" t="str">
         <v>inventory_site_modon_warehouse_ing_biryani_masala</v>
@@ -10136,10 +10136,10 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B124" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C124" t="str">
         <v>inventory_site_modon_warehouse_ing_garam_masala</v>
@@ -10201,10 +10201,10 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B125" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C125" t="str">
         <v>inventory_site_modon_warehouse_ing_italian_herbs</v>
@@ -10266,10 +10266,10 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B126" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C126" t="str">
         <v>inventory_site_modon_warehouse_ing_white_sauce_mix</v>
@@ -10331,10 +10331,10 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B127" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C127" t="str">
         <v>inventory_site_modon_warehouse_ing_chicken_stock</v>
@@ -10396,10 +10396,10 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B128" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C128" t="str">
         <v>inventory_site_modon_warehouse_ing_salt</v>
@@ -10461,10 +10461,10 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="B129" t="str">
-        <v>2026-05-03T13:12:55.453Z</v>
+        <v>2026-05-03T13:14:58.846Z</v>
       </c>
       <c r="C129" t="str">
         <v>inventory_site_modon_warehouse_ing_black_pepper</v>

</xml_diff>